<commit_message>
PHD alumini ui update
</commit_message>
<xml_diff>
--- a/excels/M-Tech_Alumini.xlsx
+++ b/excels/M-Tech_Alumini.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{544AE952-1783-45E3-9838-36EC62D15CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB475ABF-D5B7-4A95-ACFE-67599569450B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,55 +21,56 @@
     <sheet name="1972" sheetId="62" r:id="rId6"/>
     <sheet name="1974" sheetId="7" r:id="rId7"/>
     <sheet name="1975" sheetId="8" r:id="rId8"/>
-    <sheet name="1977" sheetId="9" r:id="rId9"/>
-    <sheet name="1978" sheetId="10" r:id="rId10"/>
-    <sheet name="1979" sheetId="11" r:id="rId11"/>
-    <sheet name="1980" sheetId="12" r:id="rId12"/>
-    <sheet name="1981" sheetId="13" r:id="rId13"/>
-    <sheet name="1982" sheetId="14" r:id="rId14"/>
-    <sheet name="1983" sheetId="15" r:id="rId15"/>
-    <sheet name="1984" sheetId="16" r:id="rId16"/>
-    <sheet name="1985" sheetId="17" r:id="rId17"/>
-    <sheet name="1986" sheetId="18" r:id="rId18"/>
-    <sheet name="1987" sheetId="19" r:id="rId19"/>
-    <sheet name="1988" sheetId="20" r:id="rId20"/>
-    <sheet name="1989" sheetId="21" r:id="rId21"/>
-    <sheet name="1990" sheetId="22" r:id="rId22"/>
-    <sheet name="1991" sheetId="23" r:id="rId23"/>
-    <sheet name="1992" sheetId="24" r:id="rId24"/>
-    <sheet name="1993" sheetId="25" r:id="rId25"/>
-    <sheet name="1994" sheetId="26" r:id="rId26"/>
-    <sheet name="1995" sheetId="27" r:id="rId27"/>
-    <sheet name="1996" sheetId="28" r:id="rId28"/>
-    <sheet name="1997" sheetId="29" r:id="rId29"/>
-    <sheet name="1998" sheetId="30" r:id="rId30"/>
-    <sheet name="1999" sheetId="31" r:id="rId31"/>
-    <sheet name="2000" sheetId="32" r:id="rId32"/>
-    <sheet name="2001" sheetId="33" r:id="rId33"/>
-    <sheet name="2002" sheetId="34" r:id="rId34"/>
-    <sheet name="2003" sheetId="35" r:id="rId35"/>
-    <sheet name="2004" sheetId="36" r:id="rId36"/>
-    <sheet name="2005" sheetId="37" r:id="rId37"/>
-    <sheet name="2006" sheetId="39" r:id="rId38"/>
-    <sheet name="2007" sheetId="40" r:id="rId39"/>
-    <sheet name="2008" sheetId="41" r:id="rId40"/>
-    <sheet name="2009" sheetId="42" r:id="rId41"/>
-    <sheet name="2010" sheetId="43" r:id="rId42"/>
-    <sheet name="2011" sheetId="44" r:id="rId43"/>
-    <sheet name="2012" sheetId="45" r:id="rId44"/>
-    <sheet name="2013" sheetId="46" r:id="rId45"/>
-    <sheet name="2014" sheetId="47" r:id="rId46"/>
-    <sheet name="2015" sheetId="48" r:id="rId47"/>
-    <sheet name="2016" sheetId="49" r:id="rId48"/>
-    <sheet name="2017" sheetId="50" r:id="rId49"/>
-    <sheet name="2018" sheetId="51" r:id="rId50"/>
-    <sheet name="2019" sheetId="52" r:id="rId51"/>
-    <sheet name="2020" sheetId="53" r:id="rId52"/>
-    <sheet name="2021" sheetId="54" r:id="rId53"/>
-    <sheet name="2022" sheetId="57" r:id="rId54"/>
-    <sheet name="2023" sheetId="56" r:id="rId55"/>
-    <sheet name="2024" sheetId="55" r:id="rId56"/>
-    <sheet name="2025" sheetId="58" r:id="rId57"/>
+    <sheet name="1976" sheetId="63" r:id="rId9"/>
+    <sheet name="1977" sheetId="9" r:id="rId10"/>
+    <sheet name="1978" sheetId="10" r:id="rId11"/>
+    <sheet name="1979" sheetId="11" r:id="rId12"/>
+    <sheet name="1980" sheetId="12" r:id="rId13"/>
+    <sheet name="1981" sheetId="13" r:id="rId14"/>
+    <sheet name="1982" sheetId="14" r:id="rId15"/>
+    <sheet name="1983" sheetId="15" r:id="rId16"/>
+    <sheet name="1984" sheetId="16" r:id="rId17"/>
+    <sheet name="1985" sheetId="17" r:id="rId18"/>
+    <sheet name="1986" sheetId="18" r:id="rId19"/>
+    <sheet name="1987" sheetId="19" r:id="rId20"/>
+    <sheet name="1988" sheetId="20" r:id="rId21"/>
+    <sheet name="1989" sheetId="21" r:id="rId22"/>
+    <sheet name="1990" sheetId="22" r:id="rId23"/>
+    <sheet name="1991" sheetId="23" r:id="rId24"/>
+    <sheet name="1992" sheetId="24" r:id="rId25"/>
+    <sheet name="1993" sheetId="25" r:id="rId26"/>
+    <sheet name="1994" sheetId="26" r:id="rId27"/>
+    <sheet name="1995" sheetId="27" r:id="rId28"/>
+    <sheet name="1996" sheetId="28" r:id="rId29"/>
+    <sheet name="1997" sheetId="29" r:id="rId30"/>
+    <sheet name="1998" sheetId="30" r:id="rId31"/>
+    <sheet name="1999" sheetId="31" r:id="rId32"/>
+    <sheet name="2000" sheetId="32" r:id="rId33"/>
+    <sheet name="2001" sheetId="33" r:id="rId34"/>
+    <sheet name="2002" sheetId="34" r:id="rId35"/>
+    <sheet name="2003" sheetId="35" r:id="rId36"/>
+    <sheet name="2004" sheetId="36" r:id="rId37"/>
+    <sheet name="2005" sheetId="37" r:id="rId38"/>
+    <sheet name="2006" sheetId="39" r:id="rId39"/>
+    <sheet name="2007" sheetId="40" r:id="rId40"/>
+    <sheet name="2008" sheetId="41" r:id="rId41"/>
+    <sheet name="2009" sheetId="42" r:id="rId42"/>
+    <sheet name="2010" sheetId="43" r:id="rId43"/>
+    <sheet name="2011" sheetId="44" r:id="rId44"/>
+    <sheet name="2012" sheetId="45" r:id="rId45"/>
+    <sheet name="2013" sheetId="46" r:id="rId46"/>
+    <sheet name="2014" sheetId="47" r:id="rId47"/>
+    <sheet name="2015" sheetId="48" r:id="rId48"/>
+    <sheet name="2016" sheetId="49" r:id="rId49"/>
+    <sheet name="2017" sheetId="50" r:id="rId50"/>
+    <sheet name="2018" sheetId="51" r:id="rId51"/>
+    <sheet name="2019" sheetId="52" r:id="rId52"/>
+    <sheet name="2020" sheetId="53" r:id="rId53"/>
+    <sheet name="2021" sheetId="54" r:id="rId54"/>
+    <sheet name="2022" sheetId="57" r:id="rId55"/>
+    <sheet name="2023" sheetId="56" r:id="rId56"/>
+    <sheet name="2024" sheetId="55" r:id="rId57"/>
+    <sheet name="2025" sheetId="58" r:id="rId58"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -89,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3185" uniqueCount="2679">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3193" uniqueCount="2679">
   <si>
     <t>Ramakant Jha</t>
   </si>
@@ -8601,6 +8602,87 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="69.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="88.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A1" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1762</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="12" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>160</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -8700,7 +8782,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -8784,7 +8866,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -8935,7 +9017,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -9062,7 +9144,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -14200,7 +14282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -14463,7 +14545,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -14825,7 +14907,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -15151,7 +15233,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -15360,241 +15442,6 @@
       </c>
       <c r="F16" s="12" t="s">
         <v>403</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="14.28515625" customWidth="1"/>
-    <col min="2" max="2" width="24.85546875" customWidth="1"/>
-    <col min="3" max="3" width="69" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" customWidth="1"/>
-    <col min="5" max="5" width="72.42578125" customWidth="1"/>
-    <col min="6" max="6" width="36.42578125" customWidth="1"/>
-    <col min="7" max="7" width="33.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="C2" s="13"/>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A3" s="1" t="s">
-        <v>406</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>409</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A4" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>412</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A5" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A6" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>419</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A7" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>423</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>424</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A8" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A9" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="C9" s="2"/>
-      <c r="E9" s="12" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A10" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A11" s="1" t="s">
-        <v>437</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>438</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>1736</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>439</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>440</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A12" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="C12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A13" s="1" t="s">
-        <v>444</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="E13" s="12" t="s">
-        <v>446</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A14" s="1" t="s">
-        <v>447</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>1735</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>449</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>450</v>
       </c>
     </row>
   </sheetData>
@@ -15669,6 +15516,241 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="14.28515625" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" customWidth="1"/>
+    <col min="3" max="3" width="69" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="5" max="5" width="72.42578125" customWidth="1"/>
+    <col min="6" max="6" width="36.42578125" customWidth="1"/>
+    <col min="7" max="7" width="33.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A1" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="C2" s="13"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A3" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>409</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A4" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A5" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A6" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>419</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A7" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>423</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>424</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A8" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A9" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="E9" s="12" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A10" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A11" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>1736</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>439</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>440</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A12" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A13" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="E13" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A14" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>1735</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>449</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>450</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -15916,7 +15998,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -16136,7 +16218,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -16430,7 +16512,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -16609,7 +16691,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -17853,7 +17935,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -18094,7 +18176,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -18263,7 +18345,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -23488,7 +23570,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -23729,235 +23811,6 @@
     </row>
     <row r="17" spans="8:8" ht="15.75" customHeight="1">
       <c r="H17" s="18"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col min="2" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="1">
-        <v>129701</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>738</v>
-      </c>
-      <c r="H2" s="19" t="s">
-        <v>2278</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A3" s="1">
-        <v>129702</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>739</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1663</v>
-      </c>
-      <c r="H3" s="19" t="s">
-        <v>2279</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A4" s="1">
-        <v>129703</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>740</v>
-      </c>
-      <c r="C4" t="s">
-        <v>1664</v>
-      </c>
-      <c r="H4" s="19" t="s">
-        <v>2280</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A5" s="1">
-        <v>129704</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>741</v>
-      </c>
-      <c r="H5" s="19" t="s">
-        <v>2281</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A6" s="1">
-        <v>129705</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>742</v>
-      </c>
-      <c r="C6" t="s">
-        <v>1660</v>
-      </c>
-      <c r="H6" s="19" t="s">
-        <v>2282</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A7" s="1">
-        <v>129706</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>743</v>
-      </c>
-      <c r="H7" s="19" t="s">
-        <v>2283</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A8" s="1">
-        <v>129707</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>744</v>
-      </c>
-      <c r="H8" s="19" t="s">
-        <v>2284</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A9" s="1">
-        <v>129708</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>745</v>
-      </c>
-      <c r="C9" t="s">
-        <v>1661</v>
-      </c>
-      <c r="H9" s="19" t="s">
-        <v>2285</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A10" s="1">
-        <v>129709</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>746</v>
-      </c>
-      <c r="C10" t="s">
-        <v>1665</v>
-      </c>
-      <c r="H10" s="19" t="s">
-        <v>2286</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A11" s="1">
-        <v>129710</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>747</v>
-      </c>
-      <c r="C11" t="s">
-        <v>1666</v>
-      </c>
-      <c r="H11" s="19" t="s">
-        <v>2287</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A12" s="1">
-        <v>129711</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>748</v>
-      </c>
-      <c r="C12" t="s">
-        <v>1662</v>
-      </c>
-      <c r="H12" s="19" t="s">
-        <v>2288</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A13" s="1">
-        <v>129712</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>737</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>749</v>
-      </c>
-      <c r="H13" s="19" t="s">
-        <v>2289</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A14" s="1">
-        <v>129713</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>750</v>
-      </c>
-      <c r="H14" s="19" t="s">
-        <v>2290</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A15" s="1">
-        <v>129714</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>751</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>752</v>
-      </c>
-      <c r="H15" s="19" t="s">
-        <v>2291</v>
-      </c>
-    </row>
-    <row r="23" spans="8:8" ht="15.75" customHeight="1">
-      <c r="H23" s="19" t="s">
-        <v>943</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -24050,6 +23903,235 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A1" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A2" s="1">
+        <v>129701</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="H2" s="19" t="s">
+        <v>2278</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A3" s="1">
+        <v>129702</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>739</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1663</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>2279</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A4" s="1">
+        <v>129703</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>740</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1664</v>
+      </c>
+      <c r="H4" s="19" t="s">
+        <v>2280</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A5" s="1">
+        <v>129704</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>741</v>
+      </c>
+      <c r="H5" s="19" t="s">
+        <v>2281</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A6" s="1">
+        <v>129705</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>742</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1660</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>2282</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A7" s="1">
+        <v>129706</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="H7" s="19" t="s">
+        <v>2283</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A8" s="1">
+        <v>129707</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="H8" s="19" t="s">
+        <v>2284</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A9" s="1">
+        <v>129708</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1661</v>
+      </c>
+      <c r="H9" s="19" t="s">
+        <v>2285</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A10" s="1">
+        <v>129709</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1665</v>
+      </c>
+      <c r="H10" s="19" t="s">
+        <v>2286</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A11" s="1">
+        <v>129710</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>747</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1666</v>
+      </c>
+      <c r="H11" s="19" t="s">
+        <v>2287</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A12" s="1">
+        <v>129711</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1662</v>
+      </c>
+      <c r="H12" s="19" t="s">
+        <v>2288</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A13" s="1">
+        <v>129712</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>737</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>749</v>
+      </c>
+      <c r="H13" s="19" t="s">
+        <v>2289</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A14" s="1">
+        <v>129713</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="H14" s="19" t="s">
+        <v>2290</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A15" s="1">
+        <v>129714</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>752</v>
+      </c>
+      <c r="H15" s="19" t="s">
+        <v>2291</v>
+      </c>
+    </row>
+    <row r="23" spans="8:8" ht="15.75" customHeight="1">
+      <c r="H23" s="19" t="s">
+        <v>943</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -24316,7 +24398,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -24529,7 +24611,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -24761,7 +24843,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -25071,7 +25153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -25370,7 +25452,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -25668,7 +25750,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -25976,7 +26058,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -26284,7 +26366,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -26656,410 +26738,6 @@
       </c>
       <c r="H25" s="7" t="s">
         <v>2422</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="15.75" customHeight="1">
-      <c r="B26" s="6"/>
-      <c r="C26" s="14"/>
-      <c r="H26" s="7"/>
-    </row>
-    <row r="27" spans="1:8" ht="15.75" customHeight="1">
-      <c r="B27" s="6"/>
-      <c r="C27" s="14"/>
-      <c r="H27" s="7"/>
-    </row>
-    <row r="28" spans="1:8" ht="15.75" customHeight="1">
-      <c r="B28" s="6"/>
-      <c r="C28" s="14"/>
-      <c r="H28" s="7"/>
-    </row>
-    <row r="29" spans="1:8" ht="15.75" customHeight="1">
-      <c r="B29" s="6"/>
-      <c r="C29" s="14"/>
-      <c r="H29" s="7"/>
-    </row>
-    <row r="30" spans="1:8" ht="15.75" customHeight="1">
-      <c r="B30" s="6"/>
-      <c r="C30" s="14"/>
-      <c r="H30" s="7"/>
-    </row>
-    <row r="31" spans="1:8" ht="15.75" customHeight="1">
-      <c r="B31" s="6"/>
-      <c r="C31" s="14"/>
-      <c r="H31" s="7"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2900-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:H31"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col min="2" max="2" width="36.5703125" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" t="s">
-        <v>893</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>892</v>
-      </c>
-      <c r="C2" s="14"/>
-      <c r="H2" s="7" t="s">
-        <v>2423</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A3" t="s">
-        <v>894</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>1553</v>
-      </c>
-      <c r="C3" s="14"/>
-      <c r="H3" s="7" t="s">
-        <v>2424</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A4" t="s">
-        <v>896</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>895</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>1558</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>2425</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A5" t="s">
-        <v>898</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>897</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>2141</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>2426</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A6" t="s">
-        <v>900</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>899</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>1567</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>2427</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A7" t="s">
-        <v>902</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>901</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>1557</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>2428</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A8" t="s">
-        <v>904</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>903</v>
-      </c>
-      <c r="C8" s="14"/>
-      <c r="H8" s="7" t="s">
-        <v>2429</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A9" t="s">
-        <v>906</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>905</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>1562</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>2430</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A10" t="s">
-        <v>908</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>907</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>1554</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>2431</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A11" t="s">
-        <v>910</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>909</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>1561</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>2432</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A12" t="s">
-        <v>912</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>911</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>1556</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>2433</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A13" t="s">
-        <v>914</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>913</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>2142</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>2434</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A14" t="s">
-        <v>916</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>915</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>1555</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>2435</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A15" t="s">
-        <v>918</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>917</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>2143</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>2436</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A16" t="s">
-        <v>920</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>919</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>2144</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>2437</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A17" t="s">
-        <v>922</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>921</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>1560</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>2438</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A18" t="s">
-        <v>924</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>923</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>1564</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>2439</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A19" t="s">
-        <v>926</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>925</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>1563</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>2440</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A20" t="s">
-        <v>928</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>927</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>1566</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>2441</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" t="s">
-        <v>930</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>929</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>2145</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>2442</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A22" t="s">
-        <v>932</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>931</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>1564</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>2443</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A23" t="s">
-        <v>934</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>933</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>1565</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>2444</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A24" t="s">
-        <v>936</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>935</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>2146</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>2445</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A25" t="s">
-        <v>937</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>938</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>1559</v>
-      </c>
-      <c r="H25" s="19" t="s">
-        <v>2446</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1">
@@ -27174,6 +26852,410 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2900-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="2" max="2" width="36.5703125" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A2" t="s">
+        <v>893</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="C2" s="14"/>
+      <c r="H2" s="7" t="s">
+        <v>2423</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A3" t="s">
+        <v>894</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1553</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="H3" s="7" t="s">
+        <v>2424</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A4" t="s">
+        <v>896</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>895</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>1558</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>2425</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A5" t="s">
+        <v>898</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>897</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>2141</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>2426</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A6" t="s">
+        <v>900</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>899</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>1567</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>2427</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A7" t="s">
+        <v>902</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>901</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>1557</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>2428</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A8" t="s">
+        <v>904</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C8" s="14"/>
+      <c r="H8" s="7" t="s">
+        <v>2429</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A9" t="s">
+        <v>906</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>905</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>1562</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>2430</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A10" t="s">
+        <v>908</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>907</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>1554</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>2431</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A11" t="s">
+        <v>910</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>909</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>1561</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>2432</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A12" t="s">
+        <v>912</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>911</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>1556</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>2433</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A13" t="s">
+        <v>914</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>913</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>2142</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>2434</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A14" t="s">
+        <v>916</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>915</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>1555</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>2435</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A15" t="s">
+        <v>918</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>917</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>2143</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>2436</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A16" t="s">
+        <v>920</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>919</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>2144</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>2437</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A17" t="s">
+        <v>922</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>921</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>1560</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>2438</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A18" t="s">
+        <v>924</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>923</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>1564</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>2439</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A19" t="s">
+        <v>926</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>925</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>1563</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>2440</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A20" t="s">
+        <v>928</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>927</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>1566</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>2441</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A21" t="s">
+        <v>930</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>929</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>2145</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>2442</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A22" t="s">
+        <v>932</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>931</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>1564</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>2443</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A23" t="s">
+        <v>934</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>933</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>1565</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>2444</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A24" t="s">
+        <v>936</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>935</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>2146</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>2445</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A25" t="s">
+        <v>937</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>938</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>1559</v>
+      </c>
+      <c r="H25" s="19" t="s">
+        <v>2446</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="15.75" customHeight="1">
+      <c r="B26" s="6"/>
+      <c r="C26" s="14"/>
+      <c r="H26" s="7"/>
+    </row>
+    <row r="27" spans="1:8" ht="15.75" customHeight="1">
+      <c r="B27" s="6"/>
+      <c r="C27" s="14"/>
+      <c r="H27" s="7"/>
+    </row>
+    <row r="28" spans="1:8" ht="15.75" customHeight="1">
+      <c r="B28" s="6"/>
+      <c r="C28" s="14"/>
+      <c r="H28" s="7"/>
+    </row>
+    <row r="29" spans="1:8" ht="15.75" customHeight="1">
+      <c r="B29" s="6"/>
+      <c r="C29" s="14"/>
+      <c r="H29" s="7"/>
+    </row>
+    <row r="30" spans="1:8" ht="15.75" customHeight="1">
+      <c r="B30" s="6"/>
+      <c r="C30" s="14"/>
+      <c r="H30" s="7"/>
+    </row>
+    <row r="31" spans="1:8" ht="15.75" customHeight="1">
+      <c r="B31" s="6"/>
+      <c r="C31" s="14"/>
+      <c r="H31" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2A00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -28611,7 +28693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2B00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -29085,7 +29167,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2C00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -29510,7 +29592,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2D00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -29916,7 +29998,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2E00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -30584,7 +30666,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2F00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -31002,7 +31084,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -31430,7 +31512,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -31841,7 +31923,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -32123,313 +32205,6 @@
       <c r="C26" s="14" t="s">
         <v>1822</v>
       </c>
-      <c r="H26" s="7"/>
-    </row>
-    <row r="27" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A27" s="6"/>
-      <c r="B27" s="6"/>
-      <c r="C27" s="14"/>
-      <c r="H27" s="7"/>
-    </row>
-    <row r="28" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A28" s="6"/>
-      <c r="B28" s="6"/>
-      <c r="C28" s="14"/>
-      <c r="H28" s="7"/>
-    </row>
-    <row r="29" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A29" s="6"/>
-      <c r="B29" s="6"/>
-      <c r="C29" s="14"/>
-      <c r="H29" s="7"/>
-    </row>
-    <row r="30" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6"/>
-      <c r="C30" s="14"/>
-      <c r="H30" s="7"/>
-    </row>
-    <row r="31" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A31" s="6"/>
-      <c r="B31" s="6"/>
-      <c r="C31" s="14"/>
-      <c r="H31" s="7"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3300-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:H31"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
-  <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6" t="s">
-        <v>1823</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>1824</v>
-      </c>
-      <c r="H2" s="7"/>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6" t="s">
-        <v>1825</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>1826</v>
-      </c>
-      <c r="H3" s="7"/>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6" t="s">
-        <v>1827</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>1828</v>
-      </c>
-      <c r="H4" s="7"/>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6" t="s">
-        <v>1829</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>1830</v>
-      </c>
-      <c r="H5" s="7"/>
-    </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6" t="s">
-        <v>1831</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>1832</v>
-      </c>
-      <c r="H6" s="7"/>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6" t="s">
-        <v>1833</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>1834</v>
-      </c>
-      <c r="H7" s="7"/>
-    </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6" t="s">
-        <v>1835</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>1836</v>
-      </c>
-      <c r="H8" s="7"/>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6" t="s">
-        <v>1837</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>1838</v>
-      </c>
-      <c r="H9" s="7"/>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6" t="s">
-        <v>1839</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>1840</v>
-      </c>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6" t="s">
-        <v>1841</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>1842</v>
-      </c>
-      <c r="H11" s="7"/>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6" t="s">
-        <v>1843</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>1844</v>
-      </c>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6" t="s">
-        <v>1845</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>1846</v>
-      </c>
-      <c r="H13" s="7"/>
-    </row>
-    <row r="14" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6" t="s">
-        <v>1847</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>1848</v>
-      </c>
-      <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6" t="s">
-        <v>1849</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>1850</v>
-      </c>
-      <c r="H15" s="7"/>
-    </row>
-    <row r="16" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6" t="s">
-        <v>1851</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>1852</v>
-      </c>
-      <c r="H16" s="7"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6" t="s">
-        <v>1853</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>1854</v>
-      </c>
-      <c r="H17" s="7"/>
-    </row>
-    <row r="18" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A18" s="6"/>
-      <c r="B18" s="6" t="s">
-        <v>1855</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>1856</v>
-      </c>
-      <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A19" s="6"/>
-      <c r="B19" s="6" t="s">
-        <v>1857</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>1858</v>
-      </c>
-      <c r="H19" s="7"/>
-    </row>
-    <row r="20" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A20" s="6"/>
-      <c r="B20" s="6" t="s">
-        <v>1859</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>1860</v>
-      </c>
-      <c r="H20" s="7"/>
-    </row>
-    <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" s="6"/>
-      <c r="B21" s="6" t="s">
-        <v>1861</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>1862</v>
-      </c>
-      <c r="H21" s="7"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A22" s="6"/>
-      <c r="B22" s="6" t="s">
-        <v>1863</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>1864</v>
-      </c>
-      <c r="H22" s="7"/>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A23" s="6"/>
-      <c r="B23" s="6" t="s">
-        <v>1865</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>1866</v>
-      </c>
-      <c r="H23" s="7"/>
-    </row>
-    <row r="24" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="14"/>
-      <c r="H24" s="7"/>
-    </row>
-    <row r="25" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A25" s="6"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="14"/>
-      <c r="H25" s="7"/>
-    </row>
-    <row r="26" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="14"/>
       <c r="H26" s="7"/>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1">
@@ -32543,6 +32318,313 @@
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3300-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A1" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6" t="s">
+        <v>1823</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>1824</v>
+      </c>
+      <c r="H2" s="7"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6" t="s">
+        <v>1825</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>1826</v>
+      </c>
+      <c r="H3" s="7"/>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6" t="s">
+        <v>1827</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>1828</v>
+      </c>
+      <c r="H4" s="7"/>
+    </row>
+    <row r="5" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6" t="s">
+        <v>1829</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>1830</v>
+      </c>
+      <c r="H5" s="7"/>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6" t="s">
+        <v>1831</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>1832</v>
+      </c>
+      <c r="H6" s="7"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6" t="s">
+        <v>1833</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>1834</v>
+      </c>
+      <c r="H7" s="7"/>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6" t="s">
+        <v>1835</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>1836</v>
+      </c>
+      <c r="H8" s="7"/>
+    </row>
+    <row r="9" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6" t="s">
+        <v>1837</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>1838</v>
+      </c>
+      <c r="H9" s="7"/>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6" t="s">
+        <v>1839</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>1840</v>
+      </c>
+      <c r="H10" s="7"/>
+    </row>
+    <row r="11" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6" t="s">
+        <v>1841</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>1842</v>
+      </c>
+      <c r="H11" s="7"/>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6" t="s">
+        <v>1843</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>1844</v>
+      </c>
+      <c r="H12" s="7"/>
+    </row>
+    <row r="13" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6" t="s">
+        <v>1845</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>1846</v>
+      </c>
+      <c r="H13" s="7"/>
+    </row>
+    <row r="14" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6" t="s">
+        <v>1847</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>1848</v>
+      </c>
+      <c r="H14" s="7"/>
+    </row>
+    <row r="15" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6" t="s">
+        <v>1849</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>1850</v>
+      </c>
+      <c r="H15" s="7"/>
+    </row>
+    <row r="16" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6" t="s">
+        <v>1851</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>1852</v>
+      </c>
+      <c r="H16" s="7"/>
+    </row>
+    <row r="17" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6" t="s">
+        <v>1853</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>1854</v>
+      </c>
+      <c r="H17" s="7"/>
+    </row>
+    <row r="18" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6" t="s">
+        <v>1855</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>1856</v>
+      </c>
+      <c r="H18" s="7"/>
+    </row>
+    <row r="19" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6" t="s">
+        <v>1857</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>1858</v>
+      </c>
+      <c r="H19" s="7"/>
+    </row>
+    <row r="20" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>1860</v>
+      </c>
+      <c r="H20" s="7"/>
+    </row>
+    <row r="21" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6" t="s">
+        <v>1861</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>1862</v>
+      </c>
+      <c r="H21" s="7"/>
+    </row>
+    <row r="22" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6" t="s">
+        <v>1863</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>1864</v>
+      </c>
+      <c r="H22" s="7"/>
+    </row>
+    <row r="23" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6" t="s">
+        <v>1865</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>1866</v>
+      </c>
+      <c r="H23" s="7"/>
+    </row>
+    <row r="24" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="14"/>
+      <c r="H24" s="7"/>
+    </row>
+    <row r="25" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="14"/>
+      <c r="H25" s="7"/>
+    </row>
+    <row r="26" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="14"/>
+      <c r="H26" s="7"/>
+    </row>
+    <row r="27" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="14"/>
+      <c r="H27" s="7"/>
+    </row>
+    <row r="28" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="14"/>
+      <c r="H28" s="7"/>
+    </row>
+    <row r="29" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="14"/>
+      <c r="H29" s="7"/>
+    </row>
+    <row r="30" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="14"/>
+      <c r="H30" s="7"/>
+    </row>
+    <row r="31" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="14"/>
+      <c r="H31" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -32857,7 +32939,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -33220,7 +33302,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -33546,7 +33628,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3700-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -33873,7 +33955,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3800-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -34249,7 +34331,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3900-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -34646,7 +34728,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3A00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -35431,7 +35513,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3B00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -40063,22 +40145,9 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="69.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="88.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="75" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.42578125" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEDE3C8B-AD0B-49E6-B7D6-5D3D6170558D}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
       <c r="A1" s="3" t="s">
@@ -40106,38 +40175,6 @@
         <v>140</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1762</v>
-      </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="12" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>160</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated mtech alumini data
</commit_message>
<xml_diff>
--- a/excels/M-Tech_Alumini.xlsx
+++ b/excels/M-Tech_Alumini.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB7A002-E4D4-4B71-AF31-FAE919084C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B1C557-82F7-44A6-8DDB-54DD5EFDC4D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="37" activeTab="43" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1968" sheetId="4" r:id="rId1"/>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3407" uniqueCount="2881">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3410" uniqueCount="2884">
   <si>
     <t>Ramakant Jha</t>
   </si>
@@ -8812,6 +8812,15 @@
   </si>
   <si>
     <t>The spectacular increase in the number of motor vehicles on thc road has created a social problem i.e. thc loss Of human lives through the road accidents. Road accidents have been a major social problem in thc developed countries of the world for fifty years. It only the fast decade the developing countries like India begun to experience large increase in the number Of road accidents taking place and have found it necessary to institute road safety programs. It is strongly felt that most of accidents, being a multi factor event, are not merely due to drivers fault on account of driver's negligence or ignorance of traffic rules and regulations, but also due to many other related factors such as abrupt changes in road conditions, flow characteristics, road user's behavior, climatic conditions, visibility and absence of traffic guidance, control and management devices. In the present study, the accident data of Rangareddy and Krishna districts of NH-9 from the year 2002-2006 was collected from concerned police stations in prepared data formats. data sheet covers all the accident details. At each police station First Information Reports are referred to note down the accident particulars. The analysis work has been carried out for NH-9 stretch which is passing through the Rangareddy and Krishna districts and black spots are identified.</t>
+  </si>
+  <si>
+    <t>Large  Scale production of automobile  after Second World Collored by increase in road haulage eave rize to nev requiremente for the roadø. Chio nev phenomenal transport denara created alarming accidentø on the exIEting roade. Thia accident rate io more in India vhen compared to other countrieg for every  1,OOO vehicle registered. It  nay be poøslbie to deøign the nov roado keeping oafety aapect in—view. But In the cage Of already existing roade it Ig only bad patcheø "known aa black opota" which require traffic Oafety measures. Traffic Safety equally applicable to both urban roada and rural road'. In this study the author hae gelected rural road of length 3B from bhongir to Uppal on Hyderauad — Waraneal road, for study Vith special reference to Bafety. Tvo uethoda VIZ. , Accident coefficient method and øafe coefficient method, Suggeøted by Prof. V.F.Bobkov have been applied to analyøo the rond for black spots. Accident data for yeare on the otretch collected and analyøed. It vao obøerved that there vaø a near co—roiatlon between the tvo. on tho analysis certain reconnendatlona voro node for Improvementø an the cue of noet øerlouø blackIn the Decond phage the author attempted to eøtablløh a relationghip between the accident coefficient and the Safe coefficient methods. Che idea that the safe coefficient method is easy and the expenøeø and labour Involved are minimum. In the Opinion of author ouch gtudieS are and have to be carried out on ail rural roads In Indin which enables in (1) deciding the exact black gpotg (2) fixing up priorities for improvement.</t>
+  </si>
+  <si>
+    <t>The succass of any urban transportation planning prognrnrno doponds upon accurate forecasting of diff- oront vehicles owned and operated by the residents tn the area. Mode split pmcedurog rost heavily on lcnovang the priori probability of ovmlng a particular vehicle by any Individual. A review of various methods for forecasting the vehide ovmerghip hag revealed that they either forecast the Past trend or by using statistical Nevertheless most of the behaviouNI models developed are appropriate only for a predominantly auto society and not applicable to developing economies. According-y, suitable hypothesis has been developed to replicate the Indian environment. Class Ificatdon techniques of multi— Statistical analysis was found to be an appro— priate tool for simulating multi-modal ownerships that are so common In a developing economy. Data for tlüs Investi gation were taken from Home-Interv1ew—Surveyg Of Roorkee town and Ænedabad metropolis. Attributeg responsible for deciding mode 01merghip of an individual were Identified and several models</t>
+  </si>
+  <si>
+    <t>Hyderabad is one of the major metropolitan cities Of India. By virtue OE tremendous growth in all sectors Of development such as industry, health, education etc., Hyderabad attracts trip makers not Only from the constiå;uent districts of Hyderabad region but also from places located outside its regional boundary. It is connected to other metro— poll tan cities of India by road, rail and air. In its 0'•m regional territory Che travel is mostly by buses because Of inadequate rail network and fre— In the absence of any foreseable quency of operation development in the railway network, in the next two decades bus vould remain the major mode of travel Eor the intra—regional trips For the assessment Of these future trips a scientific approach is necessary. conventional rrionage:rwfit:. breakeven Road Tranquor:C arc. tools for the will be for to c.cCabL1zh and would thia seudy an gather: Of p rezenz fro:a thc CICI (CES) and to rezplain the travel OE a Of Z direct aggregate demand model is found Ze ziraple eleg?ne for future level i z worked out. By means of loped a def:iciznc7 estimate OE nu:rber of bus at Is derivca and a recorcnenözl-.ion for correcting p resent deficiency is puefcrth. Traffic CES— tile years 1985, 1993 and 2001 t„zrked so as to enable the State Corporation (ESRTC) to estimate and crew requirements for these horizon years. region is devided into 25 traffic zones on thc population, urbanisation, agricultural and development, the transportation continuity. i*ne trips to each of these zones are calibrated usinq a package. Eased precent travel, Nyderabad City Region and City interaction Regions cru of the travel characteri *tics such trips income, coati Of travel, Hydera-b etc are studied to get a better of the causative factors. For a set of policy options, bus and pass— enger trips for the above horizon years are estimated. Some recommendations regarding further work needed in the di rection of estimation of comrnuter travel and r. i Zinc of bus stations are presented.</t>
   </si>
 </sst>
 </file>
@@ -9789,6 +9798,9 @@
       </c>
       <c r="C2" s="2" t="s">
         <v>58</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2883</v>
       </c>
       <c r="E2" s="12" t="s">
         <v>178</v>
@@ -27700,6 +27712,9 @@
       <c r="C4" s="18" t="s">
         <v>1744</v>
       </c>
+      <c r="D4" t="s">
+        <v>2881</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -41429,6 +41444,9 @@
       <c r="C2" t="s">
         <v>2879</v>
       </c>
+      <c r="D2" t="s">
+        <v>2882</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
not available text update
</commit_message>
<xml_diff>
--- a/excels/M-Tech_Alumini.xlsx
+++ b/excels/M-Tech_Alumini.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93DBEAD4-7FAC-4D86-974A-F81ECF7E114E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4AB9103-8C3F-4338-9B54-B2C6B9B0D71E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1968" sheetId="4" r:id="rId1"/>
@@ -71,7 +71,12 @@
     <sheet name="2023" sheetId="56" r:id="rId56"/>
     <sheet name="2024" sheetId="55" r:id="rId57"/>
     <sheet name="2025" sheetId="58" r:id="rId58"/>
+    <sheet name="Sheet1" sheetId="67" r:id="rId59"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="48" hidden="1">'2016'!$H$1:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="49" hidden="1">'2017'!$H$1:$H$32</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -90,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3410" uniqueCount="2884">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3504" uniqueCount="2977">
   <si>
     <t>Ramakant Jha</t>
   </si>
@@ -8821,6 +8826,285 @@
   </si>
   <si>
     <t>The success of any urban transportation planning prognrnrno doponds upon accurate forecasting of diff- oront vehicles owned and operated by the residents tn the area. Mode split pmcedurog rost heavily on lcnovang the priori probability of ovmlng a particular vehicle by any Individual. A review of various methods for forecasting the vehide ovmerghip hag revealed that they either forecast the Past trend or by using statistical Nevertheless most of the behaviouNI models developed are appropriate only for a predominantly auto society and not applicable to developing economies. According-y, suitable hypothesis has been developed to replicate the Indian environment. Class Ificatdon techniques of multi— Statistical analysis was found to be an appro— priate tool for simulating multi-modal ownerships that are so common In a developing economy. Data for tlüs Investi gation were taken from Home-Interv1ew—Surveyg Of Roorkee town and Ænedabad metropolis. Attributeg responsible for deciding mode 01merghip of an individual were Identified and several models</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Abhishek Sharma</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Akshay Kumar Kungulwar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Aravindmanikandan R</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Ganesh Rudrawar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Ganta Aslesha Prudhvi Raj</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Jayshree Chatterjee</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Vivek Manchikalapudi</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Mayank Rajak</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Polaki Appala Naidu</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Pooja Bhatt</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Rajkumar Singhal</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Sai Teja Tata</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Shashank Rajendra Dhanke</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Shrawan Kumar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Srinivas Tatipamula</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Arun Sundar Raj M P</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/Dev Inder Sharda</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2021/N Shrikar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Ramineni Rashmitha</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Abhishek Kumar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Amol Umakant Anwekar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Devendra</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Gone Sankeerthana</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Jaideep Mukherjee</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Karnati Ramya</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/K.V.N. Maheswara Raju</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Kaushik Pandey</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Shesham Koushik</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Subrat Kumar Jena</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Suyash Agrawal</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Ashar Khan</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2020/Ullam Chandu Yadav</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Akula Shyamsunder</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Bhoskar Pranav Prashant</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Cherala Shivaprasad</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Chidurala Maneesh</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Divya Gautam</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Kottur Rajkumar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Kuramana Ashok Kumar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Lanka Geethika</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Md Zabiulla</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Mewa Prasad Sahu</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/N V Neelima</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Nandala Shiva Kumar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/P. Vadde Rajasekhar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Potharaju Naveen</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Prakash Singh</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Saniga. A.M.</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/S.Surya Narayana Reddy</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Satyajit Rout</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Suhail Asger</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Suhail Rashid Vaid</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/S. Venkata Sai Tharun</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2019/Vivek Yadav</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Amit Singh</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Ankit Khatri</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Anoop Raj</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Arjun P V</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Asmita Subedi</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Ayush Kumar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/K. Vasantha Rao</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Martha Daniel</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Mohd Tahir Ansari</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Nikhil Kumar Gupta</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Pamir</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Shuddhashil Ghosh</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/S. Sudheer Kumar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/V. Sreenivasulu</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2018/Vishal Behera</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Ahmad Samir Shahsamandy</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Cherupally Santoshi</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Alok Keshari</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Attada Hareesh</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/G Vakula Devi</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Kundan Mandal</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Mahammad Sameer</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Meghna Gupta</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/M. Seshadri Naik</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Nawal Kishor Singh</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Shubham Ghosh</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Tinu Thomas</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2017/Vivek Kumar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2016/Arun Kumar Singh</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2016/Banoth Suresh</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2016/Battula Siva Babu</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2016/Bejjanki Ramesh</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2016/Geddada Niranjan</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2016/Kadagala Ramadevi</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2016/Kali Priyo Ghosal</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2016/Payal Kar</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2016/Priya Pandey</t>
+  </si>
+  <si>
+    <t>Mtech_Alumini/2016/Tapas Sau</t>
   </si>
 </sst>
 </file>
@@ -8969,7 +9253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -9042,6 +9326,18 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9328,7 +9624,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -9409,7 +9705,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -9509,7 +9805,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -9593,7 +9889,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -9748,7 +10044,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -9878,7 +10174,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -15025,7 +15321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -15291,7 +15587,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -15655,7 +15951,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -15989,7 +16285,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -16310,7 +16606,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -16545,7 +16841,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -16796,7 +17092,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -17016,7 +17312,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -17314,7 +17610,7 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -17493,7 +17789,7 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -18737,7 +19033,7 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -18984,7 +19280,7 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -19153,7 +19449,7 @@
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -24378,7 +24674,7 @@
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -24701,7 +24997,7 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -24930,7 +25226,7 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -25197,7 +25493,7 @@
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -25410,7 +25706,7 @@
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -25642,7 +25938,7 @@
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -25952,7 +26248,7 @@
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -26254,7 +26550,7 @@
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -26569,7 +26865,7 @@
 </file>
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -26896,7 +27192,7 @@
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -27213,7 +27509,7 @@
 </file>
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -27722,7 +28018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -28140,7 +28436,7 @@
 </file>
 
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -29618,7 +29914,7 @@
 </file>
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2900-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -30116,7 +30412,7 @@
 </file>
 
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2A00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -30576,7 +30872,7 @@
 </file>
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2B00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -31031,7 +31327,7 @@
 </file>
 
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2B00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2C00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -31729,14 +32025,14 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B26" r:id="rId1" display="http://mithun.cm/" xr:uid="{00000000-0004-0000-2B00-000000000000}"/>
+    <hyperlink ref="B26" r:id="rId1" display="http://mithun.cm/" xr:uid="{00000000-0004-0000-2C00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2C00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2D00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -32173,7 +32469,7 @@
 </file>
 
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2E00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -32651,7 +32947,7 @@
 </file>
 
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2E00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2F00-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -33073,14 +33369,14 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B11" r:id="rId1" display="http://ramees.pm/" xr:uid="{00000000-0004-0000-2E00-000000000000}"/>
+    <hyperlink ref="B11" r:id="rId1" display="http://ramees.pm/" xr:uid="{00000000-0004-0000-2F00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2F00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -33088,6 +33384,13 @@
   <sheetFormatPr defaultColWidth="29.140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="5.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="6.140625" customWidth="1"/>
+    <col min="7" max="7" width="8.28515625" customWidth="1"/>
+    <col min="8" max="8" width="48.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
@@ -33134,7 +33437,10 @@
       <c r="C3" s="14" t="s">
         <v>1765</v>
       </c>
-      <c r="H3" s="7"/>
+      <c r="E3" s="6"/>
+      <c r="H3" s="6" t="s">
+        <v>2967</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" customHeight="1">
       <c r="A4" s="6"/>
@@ -33144,7 +33450,9 @@
       <c r="C4" s="14" t="s">
         <v>1767</v>
       </c>
-      <c r="H4" s="7"/>
+      <c r="H4" s="6" t="s">
+        <v>2968</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1">
       <c r="A5" s="6"/>
@@ -33154,7 +33462,9 @@
       <c r="C5" s="14" t="s">
         <v>1769</v>
       </c>
-      <c r="H5" s="7"/>
+      <c r="H5" s="6" t="s">
+        <v>2969</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1">
       <c r="A6" s="6"/>
@@ -33164,7 +33474,9 @@
       <c r="C6" s="14" t="s">
         <v>1771</v>
       </c>
-      <c r="H6" s="7"/>
+      <c r="H6" s="6" t="s">
+        <v>2970</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
       <c r="A7" s="6">
@@ -33198,7 +33510,9 @@
       <c r="C9" s="14" t="s">
         <v>1777</v>
       </c>
-      <c r="H9" s="7"/>
+      <c r="H9" s="6" t="s">
+        <v>2971</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
       <c r="A10" s="6"/>
@@ -33228,7 +33542,9 @@
       <c r="C12" s="14" t="s">
         <v>1783</v>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="6" t="s">
+        <v>2972</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
       <c r="A13" s="6"/>
@@ -33238,7 +33554,9 @@
       <c r="C13" s="14" t="s">
         <v>1785</v>
       </c>
-      <c r="H13" s="7"/>
+      <c r="H13" s="6" t="s">
+        <v>2973</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1">
       <c r="A14" s="6"/>
@@ -33283,7 +33601,9 @@
       <c r="C17" s="14" t="s">
         <v>1793</v>
       </c>
-      <c r="H17" s="7"/>
+      <c r="H17" s="6" t="s">
+        <v>2974</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1">
       <c r="A18" s="6"/>
@@ -33305,7 +33625,9 @@
       <c r="C19" s="14" t="s">
         <v>1796</v>
       </c>
-      <c r="H19" s="7"/>
+      <c r="H19" s="6" t="s">
+        <v>2975</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="15.75" customHeight="1">
       <c r="A20" s="6"/>
@@ -33369,7 +33691,9 @@
       <c r="C25" s="14" t="s">
         <v>1808</v>
       </c>
-      <c r="H25" s="7"/>
+      <c r="H25" s="6" t="s">
+        <v>2976</v>
+      </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1">
       <c r="A26" s="6">
@@ -33417,6 +33741,7 @@
       <c r="H31" s="7"/>
     </row>
   </sheetData>
+  <autoFilter ref="H1:H31" xr:uid="{00000000-0009-0000-0000-000030000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -33512,12 +33837,20 @@
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H32"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" customWidth="1"/>
+    <col min="7" max="7" width="7.42578125" customWidth="1"/>
+    <col min="8" max="8" width="46.7109375" style="18" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
       <c r="A1" s="3" t="s">
@@ -33541,7 +33874,7 @@
       <c r="G1" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="3" t="s">
         <v>139</v>
       </c>
     </row>
@@ -33553,7 +33886,9 @@
       <c r="C2" s="14" t="s">
         <v>1812</v>
       </c>
-      <c r="H2" s="7"/>
+      <c r="H2" s="6" t="s">
+        <v>2954</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1">
       <c r="A3" s="6"/>
@@ -33563,7 +33898,9 @@
       <c r="C3" s="14" t="s">
         <v>1814</v>
       </c>
-      <c r="H3" s="7"/>
+      <c r="H3" s="6" t="s">
+        <v>2956</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" customHeight="1">
       <c r="A4" s="6">
@@ -33583,7 +33920,9 @@
       </c>
       <c r="F4" s="28"/>
       <c r="G4" s="28"/>
-      <c r="H4" s="7"/>
+      <c r="H4" s="6" t="s">
+        <v>2957</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1">
       <c r="A5" s="6">
@@ -33627,7 +33966,9 @@
       <c r="C7" s="14" t="s">
         <v>1822</v>
       </c>
-      <c r="H7" s="7"/>
+      <c r="H7" s="6" t="s">
+        <v>2958</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1">
       <c r="A8" s="6">
@@ -33642,7 +33983,9 @@
       <c r="D8" s="25" t="s">
         <v>2837</v>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="6" t="s">
+        <v>2955</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1">
       <c r="A9" s="6"/>
@@ -33682,7 +34025,9 @@
       <c r="C12" s="14" t="s">
         <v>1830</v>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="6" t="s">
+        <v>2959</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
       <c r="A13" s="6"/>
@@ -33692,7 +34037,9 @@
       <c r="C13" s="14" t="s">
         <v>1832</v>
       </c>
-      <c r="H13" s="7"/>
+      <c r="H13" s="6" t="s">
+        <v>2960</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1">
       <c r="A14" s="6"/>
@@ -33712,7 +34059,9 @@
       <c r="C15" s="14" t="s">
         <v>1836</v>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="6" t="s">
+        <v>2961</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1">
       <c r="A16" s="6"/>
@@ -33722,7 +34071,9 @@
       <c r="C16" s="14" t="s">
         <v>1838</v>
       </c>
-      <c r="H16" s="7"/>
+      <c r="H16" s="6" t="s">
+        <v>2962</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="15.75" customHeight="1">
       <c r="A17" s="6"/>
@@ -33732,7 +34083,9 @@
       <c r="C17" s="14" t="s">
         <v>1840</v>
       </c>
-      <c r="H17" s="7"/>
+      <c r="H17" s="6" t="s">
+        <v>2963</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1">
       <c r="A18" s="6">
@@ -33764,7 +34117,9 @@
       <c r="C20" s="14" t="s">
         <v>1846</v>
       </c>
-      <c r="H20" s="7"/>
+      <c r="H20" s="6" t="s">
+        <v>2964</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
       <c r="A21" s="6"/>
@@ -33774,7 +34129,9 @@
       <c r="C21" s="14" t="s">
         <v>1848</v>
       </c>
-      <c r="H21" s="7"/>
+      <c r="H21" s="6" t="s">
+        <v>2965</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1">
       <c r="A22" s="6"/>
@@ -33784,7 +34141,9 @@
       <c r="C22" s="14" t="s">
         <v>1850</v>
       </c>
-      <c r="H22" s="7"/>
+      <c r="H22" s="6" t="s">
+        <v>2966</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1">
       <c r="A23" s="6"/>
@@ -33855,17 +34214,22 @@
       <c r="H32" s="7"/>
     </row>
   </sheetData>
+  <autoFilter ref="H1:H32" xr:uid="{00000000-0009-0000-0000-000031000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H31"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="8" max="8" width="32.5703125" style="37" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
       <c r="A1" s="3" t="s">
@@ -33889,7 +34253,7 @@
       <c r="G1" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="34" t="s">
         <v>139</v>
       </c>
     </row>
@@ -33901,7 +34265,9 @@
       <c r="C2" s="14" t="s">
         <v>1856</v>
       </c>
-      <c r="H2" s="7"/>
+      <c r="H2" s="35" t="s">
+        <v>2939</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1">
       <c r="A3" s="6">
@@ -33916,7 +34282,9 @@
       <c r="E3" s="18" t="s">
         <v>2758</v>
       </c>
-      <c r="H3" s="7"/>
+      <c r="H3" s="35" t="s">
+        <v>2940</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" customHeight="1">
       <c r="A4" s="6">
@@ -33931,7 +34299,9 @@
       <c r="E4" s="18" t="s">
         <v>2723</v>
       </c>
-      <c r="H4" s="7"/>
+      <c r="H4" s="36" t="s">
+        <v>2941</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1">
       <c r="A5" s="6">
@@ -33946,7 +34316,9 @@
       <c r="E5" s="18" t="s">
         <v>2746</v>
       </c>
-      <c r="H5" s="7"/>
+      <c r="H5" s="36" t="s">
+        <v>2942</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1">
       <c r="A6" s="6"/>
@@ -33956,7 +34328,9 @@
       <c r="C6" s="14" t="s">
         <v>1864</v>
       </c>
-      <c r="H6" s="7"/>
+      <c r="H6" s="36" t="s">
+        <v>2943</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
       <c r="A7" s="6">
@@ -33971,7 +34345,9 @@
       <c r="E7" s="18" t="s">
         <v>2704</v>
       </c>
-      <c r="H7" s="7"/>
+      <c r="H7" s="36" t="s">
+        <v>2944</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1">
       <c r="A8" s="6"/>
@@ -33981,7 +34357,7 @@
       <c r="C8" s="14" t="s">
         <v>1868</v>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="36"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1">
       <c r="A9" s="6"/>
@@ -33991,7 +34367,7 @@
       <c r="C9" s="14" t="s">
         <v>1870</v>
       </c>
-      <c r="H9" s="7"/>
+      <c r="H9" s="36"/>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
       <c r="A10" s="6"/>
@@ -34001,7 +34377,7 @@
       <c r="C10" s="14" t="s">
         <v>1872</v>
       </c>
-      <c r="H10" s="7"/>
+      <c r="H10" s="36"/>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1">
       <c r="A11" s="6"/>
@@ -34011,7 +34387,7 @@
       <c r="C11" s="14" t="s">
         <v>1874</v>
       </c>
-      <c r="H11" s="7"/>
+      <c r="H11" s="36"/>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1">
       <c r="A12" s="6">
@@ -34026,7 +34402,7 @@
       <c r="E12" s="18" t="s">
         <v>2759</v>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="36"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
       <c r="A13" s="6">
@@ -34041,7 +34417,9 @@
       <c r="E13" s="18" t="s">
         <v>2729</v>
       </c>
-      <c r="H13" s="7"/>
+      <c r="H13" s="36" t="s">
+        <v>2945</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1">
       <c r="A14" s="6">
@@ -34056,7 +34434,9 @@
       <c r="E14" s="18" t="s">
         <v>2710</v>
       </c>
-      <c r="H14" s="7"/>
+      <c r="H14" s="36" t="s">
+        <v>2946</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="15.75" customHeight="1">
       <c r="A15" s="6">
@@ -34068,7 +34448,7 @@
       <c r="C15" s="14" t="s">
         <v>1882</v>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="36"/>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1">
       <c r="A16" s="6">
@@ -34083,7 +34463,9 @@
       <c r="E16" s="18" t="s">
         <v>2742</v>
       </c>
-      <c r="H16" s="7"/>
+      <c r="H16" s="36" t="s">
+        <v>2947</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="15.75" customHeight="1">
       <c r="A17" s="6"/>
@@ -34093,7 +34475,9 @@
       <c r="C17" s="14" t="s">
         <v>1886</v>
       </c>
-      <c r="H17" s="7"/>
+      <c r="H17" s="36" t="s">
+        <v>2948</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1">
       <c r="A18" s="6"/>
@@ -34103,7 +34487,9 @@
       <c r="C18" s="14" t="s">
         <v>1888</v>
       </c>
-      <c r="H18" s="7"/>
+      <c r="H18" s="36" t="s">
+        <v>2949</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="15.75" customHeight="1">
       <c r="A19" s="6">
@@ -34118,7 +34504,7 @@
       <c r="E19" s="18" t="s">
         <v>2760</v>
       </c>
-      <c r="H19" s="7"/>
+      <c r="H19" s="36"/>
     </row>
     <row r="20" spans="1:8" ht="15.75" customHeight="1">
       <c r="A20" s="6"/>
@@ -34128,7 +34514,7 @@
       <c r="C20" s="14" t="s">
         <v>1892</v>
       </c>
-      <c r="H20" s="7"/>
+      <c r="H20" s="36"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
       <c r="A21" s="6">
@@ -34140,7 +34526,9 @@
       <c r="C21" s="14" t="s">
         <v>1894</v>
       </c>
-      <c r="H21" s="7"/>
+      <c r="H21" s="36" t="s">
+        <v>2950</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1">
       <c r="A22" s="6"/>
@@ -34150,7 +34538,9 @@
       <c r="C22" s="14" t="s">
         <v>1896</v>
       </c>
-      <c r="H22" s="7"/>
+      <c r="H22" s="36" t="s">
+        <v>2951</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1">
       <c r="A23" s="6"/>
@@ -34160,7 +34550,9 @@
       <c r="C23" s="14" t="s">
         <v>1898</v>
       </c>
-      <c r="H23" s="7"/>
+      <c r="H23" s="36" t="s">
+        <v>2952</v>
+      </c>
     </row>
     <row r="24" spans="1:8" ht="15.75" customHeight="1">
       <c r="A24" s="6"/>
@@ -34170,7 +34562,7 @@
       <c r="C24" s="14" t="s">
         <v>1900</v>
       </c>
-      <c r="H24" s="7"/>
+      <c r="H24" s="36"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1">
       <c r="A25" s="6"/>
@@ -34180,43 +34572,45 @@
       <c r="C25" s="14" t="s">
         <v>1902</v>
       </c>
-      <c r="H25" s="7"/>
+      <c r="H25" s="36" t="s">
+        <v>2953</v>
+      </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="C26" s="14"/>
-      <c r="H26" s="7"/>
+      <c r="H26" s="36"/>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1">
       <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="14"/>
-      <c r="H27" s="7"/>
+      <c r="H27" s="36"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="14"/>
-      <c r="H28" s="7"/>
+      <c r="H28" s="36"/>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1">
       <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="14"/>
-      <c r="H29" s="7"/>
+      <c r="H29" s="36"/>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1">
       <c r="A30" s="6"/>
       <c r="B30" s="6"/>
       <c r="C30" s="14"/>
-      <c r="H30" s="7"/>
+      <c r="H30" s="36"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1">
       <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="14"/>
-      <c r="H31" s="7"/>
+      <c r="H31" s="36"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -34224,12 +34618,16 @@
 </file>
 
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:I34"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="8" max="8" width="39.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
       <c r="A1" s="3" t="s">
@@ -34290,7 +34688,9 @@
       <c r="E4" s="18" t="s">
         <v>2725</v>
       </c>
-      <c r="H4" s="7"/>
+      <c r="H4" s="6" t="s">
+        <v>2916</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1">
       <c r="A5" s="6"/>
@@ -34320,7 +34720,9 @@
       <c r="C7" s="14" t="s">
         <v>1914</v>
       </c>
-      <c r="H7" s="7"/>
+      <c r="H7" s="6" t="s">
+        <v>2917</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1">
       <c r="A8" s="6"/>
@@ -34330,7 +34732,9 @@
       <c r="C8" s="14" t="s">
         <v>1916</v>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="6" t="s">
+        <v>2918</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1">
       <c r="A9" s="6"/>
@@ -34340,7 +34744,9 @@
       <c r="C9" s="14" t="s">
         <v>1918</v>
       </c>
-      <c r="H9" s="7"/>
+      <c r="H9" s="6" t="s">
+        <v>2919</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
       <c r="A10" s="6">
@@ -34355,7 +34761,9 @@
       <c r="E10" s="18" t="s">
         <v>2741</v>
       </c>
-      <c r="H10" s="7"/>
+      <c r="H10" s="6" t="s">
+        <v>2920</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1">
       <c r="A11" s="6"/>
@@ -34375,7 +34783,9 @@
       <c r="C12" s="14" t="s">
         <v>1924</v>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="6" t="s">
+        <v>2921</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
       <c r="A13" s="6"/>
@@ -34385,7 +34795,9 @@
       <c r="C13" s="14" t="s">
         <v>1926</v>
       </c>
-      <c r="H13" s="7"/>
+      <c r="H13" s="6" t="s">
+        <v>2922</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1">
       <c r="A14" s="6"/>
@@ -34410,7 +34822,9 @@
       <c r="E15" s="18" t="s">
         <v>2740</v>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="6" t="s">
+        <v>2923</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1">
       <c r="A16" s="6"/>
@@ -34420,7 +34834,9 @@
       <c r="C16" s="14" t="s">
         <v>1932</v>
       </c>
-      <c r="H16" s="7"/>
+      <c r="H16" s="6" t="s">
+        <v>2924</v>
+      </c>
     </row>
     <row r="17" spans="1:9" ht="15.75" customHeight="1">
       <c r="A17" s="6"/>
@@ -34430,7 +34846,9 @@
       <c r="C17" s="14" t="s">
         <v>1934</v>
       </c>
-      <c r="H17" s="7"/>
+      <c r="H17" s="6" t="s">
+        <v>2925</v>
+      </c>
     </row>
     <row r="18" spans="1:9" ht="15.75" customHeight="1">
       <c r="A18" s="6">
@@ -34470,7 +34888,9 @@
       <c r="E20" s="18" t="s">
         <v>2722</v>
       </c>
-      <c r="H20" s="7"/>
+      <c r="H20" s="6" t="s">
+        <v>2926</v>
+      </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1">
       <c r="A21" s="6">
@@ -34485,7 +34905,9 @@
       <c r="E21" s="18" t="s">
         <v>2721</v>
       </c>
-      <c r="H21" s="7"/>
+      <c r="H21" s="6" t="s">
+        <v>2927</v>
+      </c>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1">
       <c r="A22" s="6"/>
@@ -34495,7 +34917,9 @@
       <c r="C22" s="14" t="s">
         <v>1944</v>
       </c>
-      <c r="H22" s="7"/>
+      <c r="H22" s="6" t="s">
+        <v>2928</v>
+      </c>
     </row>
     <row r="23" spans="1:9" ht="15.75" customHeight="1">
       <c r="A23" s="6"/>
@@ -34505,7 +34929,9 @@
       <c r="C23" s="14" t="s">
         <v>1946</v>
       </c>
-      <c r="H23" s="7"/>
+      <c r="H23" s="6" t="s">
+        <v>2929</v>
+      </c>
     </row>
     <row r="24" spans="1:9" ht="15.75" customHeight="1">
       <c r="A24" s="6">
@@ -34520,7 +34946,9 @@
       <c r="E24" s="18" t="s">
         <v>2744</v>
       </c>
-      <c r="H24" s="7"/>
+      <c r="H24" s="6" t="s">
+        <v>2930</v>
+      </c>
     </row>
     <row r="25" spans="1:9" ht="15.75" customHeight="1">
       <c r="A25" s="6"/>
@@ -34540,7 +34968,9 @@
       <c r="C26" s="14" t="s">
         <v>1952</v>
       </c>
-      <c r="H26" s="7"/>
+      <c r="H26" s="7" t="s">
+        <v>2931</v>
+      </c>
     </row>
     <row r="27" spans="1:9" ht="15.75" customHeight="1">
       <c r="A27" s="6"/>
@@ -34550,7 +34980,9 @@
       <c r="C27" s="14" t="s">
         <v>1954</v>
       </c>
-      <c r="H27" s="7"/>
+      <c r="H27" s="7" t="s">
+        <v>2932</v>
+      </c>
     </row>
     <row r="28" spans="1:9" ht="15.75" customHeight="1">
       <c r="A28" s="6"/>
@@ -34560,7 +34992,9 @@
       <c r="C28" s="14" t="s">
         <v>1956</v>
       </c>
-      <c r="H28" s="7"/>
+      <c r="H28" s="7" t="s">
+        <v>2933</v>
+      </c>
     </row>
     <row r="29" spans="1:9" ht="15.75" customHeight="1">
       <c r="A29" s="6"/>
@@ -34570,7 +35004,9 @@
       <c r="C29" s="14" t="s">
         <v>1958</v>
       </c>
-      <c r="H29" s="7"/>
+      <c r="H29" s="7" t="s">
+        <v>2934</v>
+      </c>
     </row>
     <row r="30" spans="1:9" ht="15.75" customHeight="1">
       <c r="A30" s="6"/>
@@ -34580,7 +35016,9 @@
       <c r="C30" s="14" t="s">
         <v>1960</v>
       </c>
-      <c r="H30" s="7"/>
+      <c r="H30" s="7" t="s">
+        <v>2935</v>
+      </c>
     </row>
     <row r="31" spans="1:9" ht="15.75" customHeight="1">
       <c r="A31" s="6">
@@ -34598,7 +35036,9 @@
       </c>
       <c r="F31" s="18"/>
       <c r="G31" s="18"/>
-      <c r="H31" s="1"/>
+      <c r="H31" s="1" t="s">
+        <v>2936</v>
+      </c>
       <c r="I31" s="18"/>
     </row>
     <row r="32" spans="1:9" ht="15.75" customHeight="1">
@@ -34612,7 +35052,9 @@
       <c r="E32" s="18"/>
       <c r="F32" s="18"/>
       <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
+      <c r="H32" s="18" t="s">
+        <v>2937</v>
+      </c>
       <c r="I32" s="18"/>
     </row>
     <row r="33" spans="2:9" ht="15.75" customHeight="1">
@@ -34626,7 +35068,9 @@
       <c r="E33" s="18"/>
       <c r="F33" s="18"/>
       <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
+      <c r="H33" s="18" t="s">
+        <v>2938</v>
+      </c>
       <c r="I33" s="18"/>
     </row>
     <row r="34" spans="2:9" ht="15.75" customHeight="1">
@@ -34640,7 +35084,9 @@
       <c r="E34" s="18"/>
       <c r="F34" s="18"/>
       <c r="G34" s="18"/>
-      <c r="H34" s="18"/>
+      <c r="H34" s="18" t="s">
+        <v>2937</v>
+      </c>
       <c r="I34" s="18"/>
     </row>
   </sheetData>
@@ -34649,7 +35095,7 @@
 </file>
 
 <file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -34657,6 +35103,7 @@
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="37.5703125" customWidth="1"/>
+    <col min="8" max="8" width="37.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
@@ -34693,7 +35140,9 @@
       <c r="C2" s="14" t="s">
         <v>1970</v>
       </c>
-      <c r="H2" s="7"/>
+      <c r="H2" s="7" t="s">
+        <v>2902</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1">
       <c r="A3" s="6"/>
@@ -34703,7 +35152,9 @@
       <c r="C3" s="14" t="s">
         <v>1972</v>
       </c>
-      <c r="H3" s="7"/>
+      <c r="H3" s="7" t="s">
+        <v>2903</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" customHeight="1">
       <c r="A4" s="6"/>
@@ -34713,7 +35164,7 @@
       <c r="C4" s="14" t="s">
         <v>1974</v>
       </c>
-      <c r="H4" s="7"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1">
       <c r="A5" s="6">
@@ -34725,7 +35176,9 @@
       <c r="C5" s="14" t="s">
         <v>1976</v>
       </c>
-      <c r="H5" s="7"/>
+      <c r="H5" s="7" t="s">
+        <v>2904</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1">
       <c r="A6" s="6"/>
@@ -34747,7 +35200,9 @@
       <c r="C7" s="14" t="s">
         <v>1980</v>
       </c>
-      <c r="H7" s="7"/>
+      <c r="H7" s="7" t="s">
+        <v>2905</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1">
       <c r="A8" s="6"/>
@@ -34757,7 +35212,9 @@
       <c r="C8" s="14" t="s">
         <v>1982</v>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="7" t="s">
+        <v>2906</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1">
       <c r="A9" s="6"/>
@@ -34767,7 +35224,9 @@
       <c r="C9" s="14" t="s">
         <v>1984</v>
       </c>
-      <c r="H9" s="7"/>
+      <c r="H9" s="6" t="s">
+        <v>2907</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
       <c r="A10" s="6"/>
@@ -34777,7 +35236,9 @@
       <c r="C10" s="14" t="s">
         <v>1986</v>
       </c>
-      <c r="H10" s="7"/>
+      <c r="H10" s="6" t="s">
+        <v>2908</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1">
       <c r="A11" s="6"/>
@@ -34787,7 +35248,9 @@
       <c r="C11" s="14" t="s">
         <v>1988</v>
       </c>
-      <c r="H11" s="7"/>
+      <c r="H11" s="6" t="s">
+        <v>2909</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1">
       <c r="A12" s="6"/>
@@ -34797,7 +35260,9 @@
       <c r="C12" s="14" t="s">
         <v>1990</v>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="6" t="s">
+        <v>2910</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
       <c r="A13" s="6"/>
@@ -34847,7 +35312,9 @@
       <c r="C17" s="14" t="s">
         <v>2000</v>
       </c>
-      <c r="H17" s="7"/>
+      <c r="H17" s="6" t="s">
+        <v>2911</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1">
       <c r="A18" s="6"/>
@@ -34867,7 +35334,9 @@
       <c r="C19" s="14" t="s">
         <v>2004</v>
       </c>
-      <c r="H19" s="7"/>
+      <c r="H19" s="6" t="s">
+        <v>2912</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="15.75" customHeight="1">
       <c r="A20" s="6">
@@ -34882,7 +35351,9 @@
       <c r="D20" s="18" t="s">
         <v>2734</v>
       </c>
-      <c r="H20" s="7"/>
+      <c r="H20" s="7" t="s">
+        <v>2913</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
       <c r="A21" s="6">
@@ -34930,7 +35401,9 @@
       <c r="D24" s="18" t="s">
         <v>2735</v>
       </c>
-      <c r="H24" s="7"/>
+      <c r="H24" s="6" t="s">
+        <v>2914</v>
+      </c>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1">
       <c r="A25" s="6"/>
@@ -34950,7 +35423,9 @@
       <c r="C26" s="14" t="s">
         <v>2018</v>
       </c>
-      <c r="H26" s="7"/>
+      <c r="H26" s="6" t="s">
+        <v>2915</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1">
       <c r="A27" s="6"/>
@@ -35000,6 +35475,7 @@
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="38.42578125" customWidth="1"/>
+    <col min="8" max="8" width="46.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
@@ -35036,7 +35512,9 @@
       <c r="C2" s="14" t="s">
         <v>2022</v>
       </c>
-      <c r="H2" s="7"/>
+      <c r="H2" s="1" t="s">
+        <v>2884</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1">
       <c r="A3" s="6"/>
@@ -35046,7 +35524,9 @@
       <c r="C3" s="14" t="s">
         <v>2024</v>
       </c>
-      <c r="H3" s="7"/>
+      <c r="H3" s="1" t="s">
+        <v>2885</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" customHeight="1">
       <c r="A4" s="6"/>
@@ -35056,7 +35536,9 @@
       <c r="C4" s="14" t="s">
         <v>2026</v>
       </c>
-      <c r="H4" s="7"/>
+      <c r="H4" s="6" t="s">
+        <v>2886</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1">
       <c r="A5" s="6"/>
@@ -35104,7 +35586,9 @@
       <c r="C8" s="14" t="s">
         <v>2034</v>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="6" t="s">
+        <v>2887</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1">
       <c r="A9" s="6"/>
@@ -35114,7 +35598,9 @@
       <c r="C9" s="14" t="s">
         <v>2036</v>
       </c>
-      <c r="H9" s="7"/>
+      <c r="H9" s="6" t="s">
+        <v>2888</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
       <c r="A10" s="6" t="s">
@@ -35149,7 +35635,9 @@
       <c r="C12" s="14" t="s">
         <v>2042</v>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="6" t="s">
+        <v>2889</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
       <c r="A13" s="6"/>
@@ -35169,7 +35657,9 @@
       <c r="C14" s="14" t="s">
         <v>2046</v>
       </c>
-      <c r="H14" s="7"/>
+      <c r="H14" s="6" t="s">
+        <v>2890</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="15.75" customHeight="1">
       <c r="A15" s="6"/>
@@ -35179,7 +35669,9 @@
       <c r="C15" s="14" t="s">
         <v>2048</v>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="6" t="s">
+        <v>2891</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1">
       <c r="A16" s="6" t="s">
@@ -35214,7 +35706,9 @@
       <c r="C18" s="14" t="s">
         <v>2052</v>
       </c>
-      <c r="H18" s="7"/>
+      <c r="H18" s="6" t="s">
+        <v>2892</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="15.75" customHeight="1">
       <c r="A19" s="6"/>
@@ -35224,7 +35718,9 @@
       <c r="C19" s="14" t="s">
         <v>2054</v>
       </c>
-      <c r="H19" s="7"/>
+      <c r="H19" s="6" t="s">
+        <v>2893</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="15.75" customHeight="1">
       <c r="A20" s="6"/>
@@ -35234,7 +35730,9 @@
       <c r="C20" s="14" t="s">
         <v>2056</v>
       </c>
-      <c r="H20" s="7"/>
+      <c r="H20" s="6" t="s">
+        <v>2894</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
       <c r="A21" s="6"/>
@@ -35254,7 +35752,9 @@
       <c r="C22" s="14" t="s">
         <v>2060</v>
       </c>
-      <c r="H22" s="7"/>
+      <c r="H22" s="6" t="s">
+        <v>2895</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1">
       <c r="A23" s="6"/>
@@ -35264,7 +35764,9 @@
       <c r="C23" s="14" t="s">
         <v>2062</v>
       </c>
-      <c r="H23" s="7"/>
+      <c r="H23" s="6" t="s">
+        <v>2896</v>
+      </c>
     </row>
     <row r="24" spans="1:8" ht="15.75" customHeight="1">
       <c r="A24" s="6"/>
@@ -35274,7 +35776,9 @@
       <c r="C24" s="14" t="s">
         <v>2064</v>
       </c>
-      <c r="H24" s="7"/>
+      <c r="H24" s="6" t="s">
+        <v>2897</v>
+      </c>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1">
       <c r="A25" s="6"/>
@@ -35284,7 +35788,9 @@
       <c r="C25" s="14" t="s">
         <v>2066</v>
       </c>
-      <c r="H25" s="7"/>
+      <c r="H25" s="6" t="s">
+        <v>2898</v>
+      </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1">
       <c r="A26" s="6"/>
@@ -35309,7 +35815,9 @@
       <c r="D27" s="18" t="s">
         <v>2775</v>
       </c>
-      <c r="H27" s="7"/>
+      <c r="H27" s="6" t="s">
+        <v>2899</v>
+      </c>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1">
       <c r="A28" s="6"/>
@@ -35319,7 +35827,9 @@
       <c r="C28" s="14" t="s">
         <v>2072</v>
       </c>
-      <c r="H28" s="7"/>
+      <c r="H28" s="6" t="s">
+        <v>2900</v>
+      </c>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1">
       <c r="A29" s="6" t="s">
@@ -35332,7 +35842,9 @@
         <v>2074</v>
       </c>
       <c r="D29" s="18"/>
-      <c r="H29" s="7"/>
+      <c r="H29" s="6" t="s">
+        <v>2901</v>
+      </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1">
       <c r="A30" s="6"/>
@@ -41396,8 +41908,17 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-3A00-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD7F0130-BF72-46D1-B293-8A074497C3EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -41454,7 +41975,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -41543,7 +42064,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -41705,7 +42226,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <sheetData/>

</xml_diff>